<commit_message>
adiciona dashboard financeiro em Power BI na pasta dashboard
</commit_message>
<xml_diff>
--- a/minhas_financas.xlsx
+++ b/minhas_financas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -578,6 +578,126 @@
         <v>545.9</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Lanche</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>16/06/2026</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Academia</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>11/06/2026</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Curso</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Educação</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Uber</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Transporte</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>03/06/2026</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Mercado</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Shopping</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Lazer</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>11/05/2026</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>200</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>